<commit_message>
test(#7) : CI 빌드 에러 수정
전형 외 전형을 제외한 전형으로 테스트되게 했습니다.
</commit_message>
<xml_diff>
--- a/src/test/resources/xlsx/2차전형점수.xlsx
+++ b/src/test/resources/xlsx/2차전형점수.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hsm/Documents/백엔드/haeundae-marubase/src/test/resources/xlsx/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D97F83C-C548-4C41-8432-3AE5D7874EC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC151166-4663-CF46-823C-ACFB055A5853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1440" yWindow="1140" windowWidth="21600" windowHeight="11100" xr2:uid="{7690012B-BFFA-3C48-824D-509550F219F4}"/>
   </bookViews>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="9">
   <si>
     <t>수험번호</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -89,10 +89,6 @@
   </si>
   <si>
     <t>인성영역</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>정원 외 전형</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -538,7 +534,7 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D4">
         <v>35</v>
@@ -553,7 +549,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5">
-        <v>3001</v>
+        <v>2002</v>
       </c>
       <c r="B5" t="s">
         <v>2</v>

</xml_diff>